<commit_message>
recette(suivi): hors-ligne POS rejoué + FEFO câblé → 413 OK / 5 Bloqué
Suivi du rejeu : 4 cas Bloqué débloqués (POS-10/POS-24 hors-ligne POS validé via
Playwright offline→file Dexie→resync sans doublon ; LOT-13/LOT-14 FEFO câblé+vérifié
live). Classeur passé à 413 OK / 0 KO / 5 Bloqué / 1 N/A ; +4 captures POS hors-ligne ;
synthèse mise à jour (FEFO construit, anomalie batch /pos/sales/sync signalée).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cahier_de_recettes_mini-ERP_execute_2026-06-24_main.xlsx
+++ b/Cahier_de_recettes_mini-ERP_execute_2026-06-24_main.xlsx
@@ -6450,7 +6450,7 @@
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="M26" s="37" t="inlineStr">
         <is>
-          <t>Le mode hors-ligne réel (coupure réseau + file Dexie pendingSales) n'est pas simulable de façon fiable hors navigateur instrumenté (comportement client : capture → Dexie 'pending' + idempotencyKey + reçu HTML repli). Analogue serveur vérifié : vente avec idempotencyKey générée client acceptée via POST /pos/sales/sync (status=ACCEPTED, numéro=S-2026-000040). Voir POS-11/POS-12 pour la garantie de synchro/idempotence.  [captures: POS-10-offline-banner.png, POS-10-offline-receipt.png]</t>
+          <t>[DÉBLOQUÉ — Playwright hors-ligne] Vente saisie hors-ligne (context.setOffline) → mise en file locale Dexie (1 'pending' + idempotencyKey), bandeau « Mode hors-ligne » + reçu de repli « Vente enregistrée avec succès » affichés (captures). Le mode hors-ligne est bien réel et simulable.  [captures: POS-10-offline-banner.png, POS-10_offline_banner.png, POS-10_sale_page_loaded.png, POS-10-offline-receipt.png, POS-10_offline_receipt_fallback.png]</t>
         </is>
       </c>
     </row>
@@ -7135,7 +7135,7 @@
       </c>
       <c r="J36" s="23" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="M36" s="37" t="inlineStr">
         <is>
-          <t>Le repli automatique en file locale sur erreur réseau transitoire est un comportement client (capture d'exception du POST /pos/sales → Dexie 'pending' + toast 'Vente sauvegardée localement'), non reproductible de façon fiable via API. La garantie serveur sous-jacente (idempotence + acceptation /sync sans doublon) est vérifiée (POS-11/POS-12).</t>
+          <t>[DÉBLOQUÉ — Playwright reconnexion] À la reconnexion, resynchro automatique (POST /pos/sales/sync) → l'entrée Dexie passe à 'synced' (serverSaleId présent) et le serveur a exactement 1 vente : idempotence respectée, aucun doublon. NB anomalie distincte observée : si une vente d'un lot de sync échoue (ex. no_price), tout le lot /sync part en 500 (tx rollback-only) — à durcir séparément.  [captures: POS-24_after_resync.png]</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11087,7 +11087,7 @@
     <row r="2">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>0 KO · 0 régression(s) · 9 Bloqué. Rappel : 19 KO au 2026-06-24, corrigés P0→P2 et mergés (a355ca7) — ce rejeu confirme l'état sur main.</t>
+          <t>0 KO · 0 régression(s) · 5 Bloqué. Rappel : 19 KO au 2026-06-24, corrigés P0→P2 et mergés (a355ca7) — ce rejeu confirme l'état sur main.</t>
         </is>
       </c>
     </row>
@@ -11161,7 +11161,7 @@
     <row r="7">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>LOT-13</t>
+          <t>LOT-15</t>
         </is>
       </c>
       <c r="B7" s="35" t="inlineStr">
@@ -11182,14 +11182,14 @@
       <c r="E7" s="35" t="inlineStr"/>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Non jouable: aucune route REST de consommation. La décrémentation du lot + passage EXHAUSTED + mouvement SALE_OUT passe par consumeAllocations() qui n'est PAS exposé. POST /lots/consume → HTTP 405 (route non mappée). LotController.java (vérifié sur main) ne déclare aucun endpoint de consommation; consumeAllocations n'est appelé par aucun module sortant (ventes/livraison/POS). Le pré-requis (FEFO ignore le lot épuisé) ne peut être déclenché sans flux de consommation.</t>
+          <t>[Bloqué — inchangé] La consommation FEFO AUTOMATIQUE est désormais câblée (cf. LOT-13/14), mais la SÉLECTION MANUELLE d'un lot précis (court-circuit de l'ordre FEFO) reste non exposée via l'API/UI : c'est une fonctionnalité distincte non implémentée. consumeAllocations(lotId explicite) existe au niveau SPI (testé) mais aucun écran/endpoint de vente ne permet de choisir le lot.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>LOT-14</t>
+          <t>LOT-18</t>
         </is>
       </c>
       <c r="B8" s="35" t="inlineStr">
@@ -11210,14 +11210,14 @@
       <c r="E8" s="35" t="inlineStr"/>
       <c r="F8" s="35" t="inlineStr">
         <is>
-          <t>Non jouable de bout en bout: le moteur FEFO n'est PAS branché dans le flux POS (vérifié dans LotController/code: helper /select-fefo isolé, aucune invocation côté POS/ventes/livraison). Le helper lui-même respecte l'ordre FEFO: A(exp J+7) priorisé, POST /lots/select-fefo qty 5 → HTTP 200 alloc=[{"lot":"A7","q":5}] (helperOk=true). Aucun flux POS ne l'invoque pour le valider de bout en bout.</t>
+          <t>Non déclenchable: scanExpiringLots est un job @Scheduled (cron '0 0 6 * * *') sans endpoint de déclenchement manuel (probes /lots/scan-expiring→405, /lots/alerts/scan→404, tous non mappés). Impossible d'observer de façon déterministe l'alerte [LOT-EXPIRY] dans les logs durant la session. La config d'alerte ENABLED requise existe (cf. LOT-16/17). La logique sous-jacente (findExpiringWithin filtre status ACTIVE) est validée par LOT-19.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>LOT-15</t>
+          <t>LOT-21</t>
         </is>
       </c>
       <c r="B9" s="35" t="inlineStr">
@@ -11238,19 +11238,19 @@
       <c r="E9" s="35" t="inlineStr"/>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Non jouable: la sélection manuelle de lot pour consommation passe par consumeAllocations(List&lt;LotAllocation&gt;) qui n'a aucun endpoint REST (cf. LOT-13). Le court-circuitage de FEFO par un lotId explicite ne peut donc pas être déclenché via l'API. LotController.java (main) ne déclare aucun endpoint /consume.</t>
+          <t>Non déclenchable: markExpiredLots est un job @Scheduled (cron '0 30 6 * * *') exécutant markExpiredLotsBeforeDate (UPDATE status=EXPIRED WHERE expirationDate&lt;today AND status=ACTIVE). Aucun endpoint manuel (probe /lots/mark-expired→405 non mappé). Preuve qu'il n'a pas tourné en session: un lot créé à exp=hier reste status=ACTIVE (ACTIVE) au lieu d'EXPIRED. La requête de marquage existe et est validée par LOT-19/20 (filtre status).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>LOT-18</t>
+          <t>BRC-17</t>
         </is>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="C10" s="35" t="inlineStr">
@@ -11266,119 +11266,7 @@
       <c r="E10" s="35" t="inlineStr"/>
       <c r="F10" s="35" t="inlineStr">
         <is>
-          <t>Non déclenchable: scanExpiringLots est un job @Scheduled (cron '0 0 6 * * *') sans endpoint de déclenchement manuel (probes /lots/scan-expiring→405, /lots/alerts/scan→404, tous non mappés). Impossible d'observer de façon déterministe l'alerte [LOT-EXPIRY] dans les logs durant la session. La config d'alerte ENABLED requise existe (cf. LOT-16/17). La logique sous-jacente (findExpiringWithin filtre status ACTIVE) est validée par LOT-19.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>LOT-21</t>
-        </is>
-      </c>
-      <c r="B11" s="35" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="C11" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D11" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E11" s="35" t="inlineStr"/>
-      <c r="F11" s="35" t="inlineStr">
-        <is>
-          <t>Non déclenchable: markExpiredLots est un job @Scheduled (cron '0 30 6 * * *') exécutant markExpiredLotsBeforeDate (UPDATE status=EXPIRED WHERE expirationDate&lt;today AND status=ACTIVE). Aucun endpoint manuel (probe /lots/mark-expired→405 non mappé). Preuve qu'il n'a pas tourné en session: un lot créé à exp=hier reste status=ACTIVE (ACTIVE) au lieu d'EXPIRED. La requête de marquage existe et est validée par LOT-19/20 (filtre status).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>BRC-17</t>
-        </is>
-      </c>
-      <c r="B12" s="35" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="C12" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D12" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E12" s="35" t="inlineStr"/>
-      <c r="F12" s="35" t="inlineStr">
-        <is>
           <t>Chemin error.reception.already_posted non atteignable via l'API publique : POST /record fixe TOUJOURS le bon à RECEIVED (statut terminal). Tentative de déblocage: record partiel 2/4 sur un BRC IN_PROGRESS -&gt; statut=RECEIVED ; cancel ensuite -&gt; 422 code=error.reception.already_received (already_received, jamais already_posted). La garde existe (GoodsReceiptService) mais n'est pas déclenchable par le flux normal record-&gt;cancel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>POS-10</t>
-        </is>
-      </c>
-      <c r="B13" s="35" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="C13" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D13" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E13" s="35" t="inlineStr"/>
-      <c r="F13" s="35" t="inlineStr">
-        <is>
-          <t>Le mode hors-ligne réel (coupure réseau + file Dexie pendingSales) n'est pas simulable de façon fiable hors navigateur instrumenté (comportement client : capture → Dexie 'pending' + idempotencyKey + reçu HTML repli). Analogue serveur vérifié : vente avec idempotencyKey générée client acceptée via POST /pos/sales/sync (status=ACCEPTED, numéro=S-2026-000040). Voir POS-11/POS-12 pour la garantie de synchro/idempotence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>POS-24</t>
-        </is>
-      </c>
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D14" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E14" s="35" t="inlineStr"/>
-      <c r="F14" s="35" t="inlineStr">
-        <is>
-          <t>Le repli automatique en file locale sur erreur réseau transitoire est un comportement client (capture d'exception du POST /pos/sales → Dexie 'pending' + toast 'Vente sauvegardée localement'), non reproductible de façon fiable via API. La garantie serveur sous-jacente (idempotence + acceptation /sync sans doublon) est vérifiée (POS-11/POS-12).</t>
         </is>
       </c>
     </row>
@@ -12037,7 +11925,7 @@
       </c>
       <c r="M10" s="37" t="inlineStr">
         <is>
-          <t>[API] Non testable end-to-end (inchangé vs 2026-06-24) : le seul super-admin disponible (root@minierp.local) est membre du tenant 'demo' uniquement et n'est rattaché à aucun tenant suspendable jetable -&gt; login de root sur le code du tenant SUSPENDED = 401 auth.bad_credentials (non-membre, pas un blocage de statut), et aucun endpoint API ne permet de poser is_super_admin sur un user jetable. Le profil root confirme isSuperAdmin=true (rôle SUPER_ADMIN). Le contournement ensureTenantLoggable pour super-admin est corroboré par AUTH-07 (un user standard du MÊME tenant suspendu est bien bloqué en 403).  [VÉRIF] Débloqué (promotion super-admin via DB) : sur un tenant SUSPENDED, l'admin standard → 403 auth.tenant_suspended, mais le même user promu super_admin → 200 (roles [SUPER_ADMIN,TENANT_ADMIN]). Le contournement super-admin est confirmé.</t>
+          <t>[VÉRIF] Débloqué (promotion super-admin via DB) : sur un tenant SUSPENDED, l'admin standard → 403 auth.tenant_suspended, mais le même user promu super_admin → 200 (roles [SUPER_ADMIN,TENANT_ADMIN]). Le contournement super-admin est confirmé.</t>
         </is>
       </c>
     </row>
@@ -24431,7 +24319,7 @@
       </c>
       <c r="J15" s="20" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K15" s="20" t="inlineStr">
@@ -24446,7 +24334,7 @@
       </c>
       <c r="M15" s="36" t="inlineStr">
         <is>
-          <t>Non jouable: aucune route REST de consommation. La décrémentation du lot + passage EXHAUSTED + mouvement SALE_OUT passe par consumeAllocations() qui n'est PAS exposé. POST /lots/consume → HTTP 405 (route non mappée). LotController.java (vérifié sur main) ne déclare aucun endpoint de consommation; consumeAllocations n'est appelé par aucun module sortant (ventes/livraison/POS). Le pré-requis (FEFO ignore le lot épuisé) ne peut être déclenché sans flux de consommation.</t>
+          <t>[DÉBLOQUÉ — FEFO câblé + vérifié live] La consommation FEFO est désormais branchée dans la vente/livraison/POS (LotOperations.consumeFefoIfTracked appelé par DeliveryService et PosService). Vente POS de 7 sur un produit à lots (A exp 2026-07-15 qty5, B exp 2026-12-31 qty10) → lot A passe à 0/EXHAUSTED, mouvement SALE_OUT enregistré, B décrémenté à 8. Plus de chemin mort.</t>
         </is>
       </c>
     </row>
@@ -24500,7 +24388,7 @@
       </c>
       <c r="J16" s="23" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr">
@@ -24515,7 +24403,7 @@
       </c>
       <c r="M16" s="37" t="inlineStr">
         <is>
-          <t>Non jouable de bout en bout: le moteur FEFO n'est PAS branché dans le flux POS (vérifié dans LotController/code: helper /select-fefo isolé, aucune invocation côté POS/ventes/livraison). Le helper lui-même respecte l'ordre FEFO: A(exp J+7) priorisé, POST /lots/select-fefo qty 5 → HTTP 200 alloc=[{"lot":"A7","q":5}] (helperOk=true). Aucun flux POS ne l'invoque pour le valider de bout en bout.</t>
+          <t>[DÉBLOQUÉ — FEFO câblé + vérifié live] FEFO automatique branché en encaissement POS (PosService.createSale → consumeFefoIfTracked, couvre aussi la resync hors-ligne). Ordre FEFO confirmé en live : le lot le plus proche de péremption (A) est consommé avant B (A 5→0, B 10→8). La NB du cas (« pas branché de bout en bout ») est levée. 133 IT verts (3 nouveaux tests FEFO).</t>
         </is>
       </c>
     </row>
@@ -24584,7 +24472,7 @@
       </c>
       <c r="M17" s="36" t="inlineStr">
         <is>
-          <t>Non jouable: la sélection manuelle de lot pour consommation passe par consumeAllocations(List&lt;LotAllocation&gt;) qui n'a aucun endpoint REST (cf. LOT-13). Le court-circuitage de FEFO par un lotId explicite ne peut donc pas être déclenché via l'API. LotController.java (main) ne déclare aucun endpoint /consume.</t>
+          <t>[Bloqué — inchangé] La consommation FEFO AUTOMATIQUE est désormais câblée (cf. LOT-13/14), mais la SÉLECTION MANUELLE d'un lot précis (court-circuit de l'ordre FEFO) reste non exposée via l'API/UI : c'est une fonctionnalité distincte non implémentée. consumeAllocations(lotId explicite) existe au niveau SPI (testé) mais aucun écran/endpoint de vente ne permet de choisir le lot.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
recette(suivi 2): jobs planifiés débloqués via endpoints temporaires → 416 OK / 2 Bloqué
LOT-18/LOT-21/TEN-11 vérifiés via les déclencheurs temporaires → OK. Classeur à
416 OK / 0 KO / 2 Bloqué / 1 N/A ; il ne reste Bloqué que LOT-15 (sélection manuelle
de lot) et BRC-17 (garde inatteignable). Synthèse mise à jour (Suivi 2 + fix POS sync).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cahier_de_recettes_mini-ERP_execute_2026-06-24_main.xlsx
+++ b/Cahier_de_recettes_mini-ERP_execute_2026-06-24_main.xlsx
@@ -7150,7 +7150,7 @@
       </c>
       <c r="M36" s="37" t="inlineStr">
         <is>
-          <t>[DÉBLOQUÉ — Playwright reconnexion] À la reconnexion, resynchro automatique (POST /pos/sales/sync) → l'entrée Dexie passe à 'synced' (serverSaleId présent) et le serveur a exactement 1 vente : idempotence respectée, aucun doublon. NB anomalie distincte observée : si une vente d'un lot de sync échoue (ex. no_price), tout le lot /sync part en 500 (tx rollback-only) — à durcir séparément.  [captures: POS-24_after_resync.png]</t>
+          <t>[DÉBLOQUÉ — Playwright reconnexion] À la reconnexion, resynchro automatique (POST /pos/sales/sync) → l'entrée Dexie passe à 'synced' (serverSaleId présent) et le serveur a exactement 1 vente : idempotence respectée, aucun doublon. NB anomalie distincte CORRIGÉE depuis : le batch /pos/sales/sync est désormais isolé par vente (une vente fautive ne fait plus 500 tout le lot).  [captures: POS-24_after_resync.png]</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11087,7 +11087,7 @@
     <row r="2">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>0 KO · 0 régression(s) · 5 Bloqué. Rappel : 19 KO au 2026-06-24, corrigés P0→P2 et mergés (a355ca7) — ce rejeu confirme l'état sur main.</t>
+          <t>0 KO · 0 régression(s) · 2 Bloqué. Rappel : 19 KO au 2026-06-24, corrigés P0→P2 et mergés (a355ca7) — ce rejeu confirme l'état sur main.</t>
         </is>
       </c>
     </row>
@@ -11133,12 +11133,12 @@
     <row r="6">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>TEN-11</t>
+          <t>LOT-15</t>
         </is>
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="C6" s="35" t="inlineStr">
@@ -11154,19 +11154,19 @@
       <c r="E6" s="35" t="inlineStr"/>
       <c r="F6" s="35" t="inlineStr">
         <is>
-          <t>[—] Inchangé vs 2026-06-24 : le job planifié TenantExpiryJob.sweep() (cron 07:00) n'a aucun endpoint d'API de déclenchement manuel (probes /jobs/tenant-expiry/run, /organizations/sweep-expiry, /admin/jobs/tenant-expiry -&gt; 404/405), et la fenêtre de grâce/expiration n'est pas simulable via l'API (pas d'écriture directe trialEndsAt/pastDueSince). Non exécutable dans ce harnais sans accès DB hors-API. Effet indirect cohérent : 'demo' est en PAST_DUE/Impayé (audit ORG_PAST_DUE).</t>
+          <t>[Bloqué — inchangé] La consommation FEFO AUTOMATIQUE est désormais câblée (cf. LOT-13/14), mais la SÉLECTION MANUELLE d'un lot précis (court-circuit de l'ordre FEFO) reste non exposée via l'API/UI : c'est une fonctionnalité distincte non implémentée. consumeAllocations(lotId explicite) existe au niveau SPI (testé) mais aucun écran/endpoint de vente ne permet de choisir le lot.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>LOT-15</t>
+          <t>BRC-17</t>
         </is>
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="C7" s="35" t="inlineStr">
@@ -11181,90 +11181,6 @@
       </c>
       <c r="E7" s="35" t="inlineStr"/>
       <c r="F7" s="35" t="inlineStr">
-        <is>
-          <t>[Bloqué — inchangé] La consommation FEFO AUTOMATIQUE est désormais câblée (cf. LOT-13/14), mais la SÉLECTION MANUELLE d'un lot précis (court-circuit de l'ordre FEFO) reste non exposée via l'API/UI : c'est une fonctionnalité distincte non implémentée. consumeAllocations(lotId explicite) existe au niveau SPI (testé) mais aucun écran/endpoint de vente ne permet de choisir le lot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="35" t="inlineStr">
-        <is>
-          <t>LOT-18</t>
-        </is>
-      </c>
-      <c r="B8" s="35" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="C8" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D8" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E8" s="35" t="inlineStr"/>
-      <c r="F8" s="35" t="inlineStr">
-        <is>
-          <t>Non déclenchable: scanExpiringLots est un job @Scheduled (cron '0 0 6 * * *') sans endpoint de déclenchement manuel (probes /lots/scan-expiring→405, /lots/alerts/scan→404, tous non mappés). Impossible d'observer de façon déterministe l'alerte [LOT-EXPIRY] dans les logs durant la session. La config d'alerte ENABLED requise existe (cf. LOT-16/17). La logique sous-jacente (findExpiringWithin filtre status ACTIVE) est validée par LOT-19.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>LOT-21</t>
-        </is>
-      </c>
-      <c r="B9" s="35" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D9" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E9" s="35" t="inlineStr"/>
-      <c r="F9" s="35" t="inlineStr">
-        <is>
-          <t>Non déclenchable: markExpiredLots est un job @Scheduled (cron '0 30 6 * * *') exécutant markExpiredLotsBeforeDate (UPDATE status=EXPIRED WHERE expirationDate&lt;today AND status=ACTIVE). Aucun endpoint manuel (probe /lots/mark-expired→405 non mappé). Preuve qu'il n'a pas tourné en session: un lot créé à exp=hier reste status=ACTIVE (ACTIVE) au lieu d'EXPIRED. La requête de marquage existe et est validée par LOT-19/20 (filtre status).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>BRC-17</t>
-        </is>
-      </c>
-      <c r="B10" s="35" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="C10" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D10" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E10" s="35" t="inlineStr"/>
-      <c r="F10" s="35" t="inlineStr">
         <is>
           <t>Chemin error.reception.already_posted non atteignable via l'API publique : POST /record fixe TOUJOURS le bon à RECEIVED (statut terminal). Tentative de déblocage: record partiel 2/4 sur un BRC IN_PROGRESS -&gt; statut=RECEIVED ; cancel ensuite -&gt; 422 code=error.reception.already_received (already_received, jamais already_posted). La garde existe (GoodsReceiptService) mais n'est pas déclenchable par le flux normal record-&gt;cancel.</t>
         </is>
@@ -13612,7 +13528,7 @@
       </c>
       <c r="J35" s="20" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K35" s="20" t="inlineStr">
@@ -13627,7 +13543,7 @@
       </c>
       <c r="M35" s="36" t="inlineStr">
         <is>
-          <t>[—] Inchangé vs 2026-06-24 : le job planifié TenantExpiryJob.sweep() (cron 07:00) n'a aucun endpoint d'API de déclenchement manuel (probes /jobs/tenant-expiry/run, /organizations/sweep-expiry, /admin/jobs/tenant-expiry -&gt; 404/405), et la fenêtre de grâce/expiration n'est pas simulable via l'API (pas d'écriture directe trialEndsAt/pastDueSince). Non exécutable dans ce harnais sans accès DB hors-API. Effet indirect cohérent : 'demo' est en PAST_DUE/Impayé (audit ORG_PAST_DUE).</t>
+          <t>[DÉBLOQUÉ — endpoint de déclenchement temporaire] Job @Scheduled TenantExpiryJob.sweep (grâce→suspension, cron 0 0 7) rendu déclenchable via POST /api/v1/dev/jobs/tenants/expiry-sweep (TEMPORAIRE, @Profile('!prod'), super-admin uniquement). Vérifié live : tenant PAST_DUE depuis &gt; grâce (7j) → après sweep, statut SUSPENDED ; un tenant-admin reçoit 403 (garde super-admin OK).</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24579,7 @@
       </c>
       <c r="J20" s="23" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr">
@@ -24678,7 +24594,7 @@
       </c>
       <c r="M20" s="37" t="inlineStr">
         <is>
-          <t>Non déclenchable: scanExpiringLots est un job @Scheduled (cron '0 0 6 * * *') sans endpoint de déclenchement manuel (probes /lots/scan-expiring→405, /lots/alerts/scan→404, tous non mappés). Impossible d'observer de façon déterministe l'alerte [LOT-EXPIRY] dans les logs durant la session. La config d'alerte ENABLED requise existe (cf. LOT-16/17). La logique sous-jacente (findExpiringWithin filtre status ACTIVE) est validée par LOT-19.</t>
+          <t>[DÉBLOQUÉ — endpoint de déclenchement temporaire] Job @Scheduled scanExpiringLots (alertes, cron 0 0 6) rendu déclenchable via POST /api/v1/dev/jobs/lots/scan-expiring (TEMPORAIRE, @Profile('!prod'), à retirer avant prod). Vérifié live : config d'alerte activée + lot proche de péremption → HTTP 200, alerte [LOT-EXPIRY] WARNING émise dans les logs serveur. Même logique que le planificateur.</t>
         </is>
       </c>
     </row>
@@ -24869,7 +24785,7 @@
       </c>
       <c r="J23" s="20" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K23" s="20" t="inlineStr">
@@ -24884,7 +24800,7 @@
       </c>
       <c r="M23" s="36" t="inlineStr">
         <is>
-          <t>Non déclenchable: markExpiredLots est un job @Scheduled (cron '0 30 6 * * *') exécutant markExpiredLotsBeforeDate (UPDATE status=EXPIRED WHERE expirationDate&lt;today AND status=ACTIVE). Aucun endpoint manuel (probe /lots/mark-expired→405 non mappé). Preuve qu'il n'a pas tourné en session: un lot créé à exp=hier reste status=ACTIVE (ACTIVE) au lieu d'EXPIRED. La requête de marquage existe et est validée par LOT-19/20 (filtre status).</t>
+          <t>[DÉBLOQUÉ — endpoint de déclenchement temporaire] Job @Scheduled markExpiredLots (passage EXPIRED, cron 0 30 6) rendu déclenchable via POST /api/v1/dev/jobs/lots/mark-expired (TEMPORAIRE, @Profile('!prod')). Vérifié live : lot ACTIVE à péremption passée → après déclenchement, statut EXPIRED (ACTIVE→EXPIRED confirmé en DB).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
recette(suivi 3): sélection manuelle de lot implémentée → 417 OK / 1 Bloqué
LOT-15 vérifié → OK. Classeur à 417 OK / 0 KO / 1 Bloqué / 1 N/A ; il ne reste Bloqué
que BRC-17 (garde inatteignable via l'API). Synthèse mise à jour (Suivi 3).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cahier_de_recettes_mini-ERP_execute_2026-06-24_main.xlsx
+++ b/Cahier_de_recettes_mini-ERP_execute_2026-06-24_main.xlsx
@@ -11066,7 +11066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11087,7 +11087,7 @@
     <row r="2">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>0 KO · 0 régression(s) · 2 Bloqué. Rappel : 19 KO au 2026-06-24, corrigés P0→P2 et mergés (a355ca7) — ce rejeu confirme l'état sur main.</t>
+          <t>0 KO · 0 régression(s) · 1 Bloqué. Rappel : 19 KO au 2026-06-24, corrigés P0→P2 et mergés (a355ca7) — ce rejeu confirme l'état sur main.</t>
         </is>
       </c>
     </row>
@@ -11133,12 +11133,12 @@
     <row r="6">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>LOT-15</t>
+          <t>BRC-17</t>
         </is>
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="C6" s="35" t="inlineStr">
@@ -11153,34 +11153,6 @@
       </c>
       <c r="E6" s="35" t="inlineStr"/>
       <c r="F6" s="35" t="inlineStr">
-        <is>
-          <t>[Bloqué — inchangé] La consommation FEFO AUTOMATIQUE est désormais câblée (cf. LOT-13/14), mais la SÉLECTION MANUELLE d'un lot précis (court-circuit de l'ordre FEFO) reste non exposée via l'API/UI : c'est une fonctionnalité distincte non implémentée. consumeAllocations(lotId explicite) existe au niveau SPI (testé) mais aucun écran/endpoint de vente ne permet de choisir le lot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="35" t="inlineStr">
-        <is>
-          <t>BRC-17</t>
-        </is>
-      </c>
-      <c r="B7" s="35" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="C7" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="D7" s="35" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="E7" s="35" t="inlineStr"/>
-      <c r="F7" s="35" t="inlineStr">
         <is>
           <t>Chemin error.reception.already_posted non atteignable via l'API publique : POST /record fixe TOUJOURS le bon à RECEIVED (statut terminal). Tentative de déblocage: record partiel 2/4 sur un BRC IN_PROGRESS -&gt; statut=RECEIVED ; cancel ensuite -&gt; 422 code=error.reception.already_received (already_received, jamais already_posted). La garde existe (GoodsReceiptService) mais n'est pas déclenchable par le flux normal record-&gt;cancel.</t>
         </is>
@@ -24373,7 +24345,7 @@
       </c>
       <c r="J17" s="20" t="inlineStr">
         <is>
-          <t>Bloqué</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="K17" s="20" t="inlineStr">
@@ -24388,7 +24360,7 @@
       </c>
       <c r="M17" s="36" t="inlineStr">
         <is>
-          <t>[Bloqué — inchangé] La consommation FEFO AUTOMATIQUE est désormais câblée (cf. LOT-13/14), mais la SÉLECTION MANUELLE d'un lot précis (court-circuit de l'ordre FEFO) reste non exposée via l'API/UI : c'est une fonctionnalité distincte non implémentée. consumeAllocations(lotId explicite) existe au niveau SPI (testé) mais aucun écran/endpoint de vente ne permet de choisir le lot.</t>
+          <t>[IMPLÉMENTÉ + vérifié live] La sélection MANUELLE d'un lot est désormais possible : la ligne de vente POS accepte un champ lotAllocations [{lotId, quantity}] qui court-circuite FEFO. Nouveau SPI consumeExplicitLots (valide : lot ACTIVE du bon variant/entrepôt, quantité suffisante, somme == qté de la ligne ; sinon 422). Vérifié live : vente ciblant le lot à péremption la PLUS LOINTAINE → ce lot décrémente (10→6), le lot FEFO le plus proche reste intact (5) ; allocations incohérentes → 422 error.lot.allocation_qty_mismatch. 137 IT verts (3 nouveaux tests).</t>
         </is>
       </c>
     </row>

</xml_diff>